<commit_message>
added cross target runs to run list
</commit_message>
<xml_diff>
--- a/GEp5 GOOD RUN LIST_ps12_filtered.xlsx
+++ b/GEp5 GOOD RUN LIST_ps12_filtered.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/spaubt/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/spaubt/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46D40822-EA4F-FC4F-876F-FFF2996A0FA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CE62591-B89D-7D47-B084-5E5DC289DD0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="160" yWindow="740" windowWidth="14940" windowHeight="16720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="55560" yWindow="1300" windowWidth="21280" windowHeight="22000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="replayed runs" sheetId="3" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="106">
   <si>
     <t>Q^2=11.109</t>
   </si>
@@ -336,28 +336,16 @@
     <t>Replaying</t>
   </si>
   <si>
-    <t>bold runs have ref signal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">timing peak (ns) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">4140 check on the side </t>
-  </si>
-  <si>
-    <t>4139 check on side</t>
-  </si>
-  <si>
-    <t>4344 maybe probelmatic</t>
-  </si>
-  <si>
-    <t>&lt;- Not replayed</t>
-  </si>
-  <si>
     <t>Good Run Number</t>
   </si>
   <si>
     <t>Bad Run Number</t>
+  </si>
+  <si>
+    <t>timing peak before offsets (ns)</t>
+  </si>
+  <si>
+    <t>other</t>
   </si>
 </sst>
 </file>
@@ -368,11 +356,18 @@
     <numFmt numFmtId="164" formatCode="hh&quot;:&quot;mm"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
     <numFmt numFmtId="166" formatCode="m/d/yyyy"/>
-    <numFmt numFmtId="168" formatCode="mm/dd/yyyy"/>
+    <numFmt numFmtId="167" formatCode="mm/dd/yyyy"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -417,8 +412,28 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
+      <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Helvetica Neue"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Helvetica Neue"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -516,208 +531,212 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="99">
+  <cellXfs count="103">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="2" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="165" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="11" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="11" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="11" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="11" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="166" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="6" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="167" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="9" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="20" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="20" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="9" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="9" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="4" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="4" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="4" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="9" fontId="4" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="4" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="20" fontId="4" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="9" fontId="4" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="4" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="9" fontId="4" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="4" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="166" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="2" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="6" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="6" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="2" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="6" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="168" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="9" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="20" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="4" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="166" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="20" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="9" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="166" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="9" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="2" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="166" fontId="3" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="3" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="2" fontId="3" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="166" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="9" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="2" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="166" fontId="3" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="20" fontId="3" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="9" fontId="3" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="2" fontId="3" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="166" fontId="3" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="9" fontId="3" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="2" fontId="3" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="166" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="166" fontId="5" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="2" fontId="5" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="9" fontId="4" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="4" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="166" fontId="3" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="9" fontId="3" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="2" fontId="3" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1020,307 +1039,572 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{47B1887D-CAA8-C44D-89EA-6CFDDC16C982}">
-  <dimension ref="A1:H43"/>
+  <dimension ref="A1:F52"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.83203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="B1" t="s">
+        <v>104</v>
+      </c>
+      <c r="C1" t="s">
         <v>103</v>
-      </c>
-      <c r="C1" t="s">
-        <v>109</v>
       </c>
       <c r="E1" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2">
+      <c r="F1" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A2" s="100">
         <v>3573</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="100">
         <v>30</v>
       </c>
       <c r="C2">
+        <v>3574</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A3" s="100">
+        <v>3575</v>
+      </c>
+      <c r="B3" s="100">
+        <v>30</v>
+      </c>
+      <c r="C3" s="100">
         <v>3601</v>
       </c>
-      <c r="E2">
-        <v>3574</v>
-      </c>
-      <c r="F2" t="s">
-        <v>107</v>
-      </c>
-      <c r="H2" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="C3" s="98"/>
-      <c r="E3">
-        <v>3573</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A4">
-        <v>3575</v>
-      </c>
-      <c r="B4">
-        <v>30</v>
-      </c>
-      <c r="F4">
-        <v>3601</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="F5">
+    </row>
+    <row r="4" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A4" s="101">
         <v>3602</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="F6">
+      <c r="B4" s="101">
+        <v>34.906300000000002</v>
+      </c>
+      <c r="C4" s="100">
+        <v>3623</v>
+      </c>
+      <c r="E4" s="98"/>
+      <c r="F4" s="99"/>
+    </row>
+    <row r="5" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A5" s="101">
         <v>3603</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="E7">
+      <c r="B5" s="101">
+        <v>34.995899999999999</v>
+      </c>
+      <c r="C5" s="100">
+        <v>3684</v>
+      </c>
+      <c r="E5" s="98"/>
+      <c r="F5" s="99"/>
+    </row>
+    <row r="6" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A6" s="101">
         <v>3604</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="E8">
-        <v>3623</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="E9">
+      <c r="B6" s="101">
+        <v>34.999600000000001</v>
+      </c>
+      <c r="C6" s="100">
+        <v>3773</v>
+      </c>
+      <c r="E6" s="98"/>
+      <c r="F6" s="99"/>
+    </row>
+    <row r="7" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A7" s="101">
         <v>3648</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="E10">
+      <c r="B7" s="101">
+        <v>34.718200000000003</v>
+      </c>
+      <c r="C7" s="100">
+        <v>3774</v>
+      </c>
+      <c r="E7" s="98"/>
+      <c r="F7" s="99"/>
+    </row>
+    <row r="8" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A8" s="101">
         <v>3682</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="E11">
-        <v>3684</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="E12">
+      <c r="B8" s="101">
+        <v>34.308599999999998</v>
+      </c>
+      <c r="C8" s="100">
+        <v>4139</v>
+      </c>
+      <c r="E8" s="98"/>
+      <c r="F8" s="99"/>
+    </row>
+    <row r="9" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A9" s="101">
         <v>3685</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="E13">
+      <c r="B9" s="101">
+        <v>34.210099999999997</v>
+      </c>
+      <c r="C9" s="100">
+        <v>4140</v>
+      </c>
+      <c r="E9" s="98"/>
+      <c r="F9" s="99"/>
+    </row>
+    <row r="10" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A10" s="101">
         <v>3686</v>
       </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="E14">
+      <c r="B10" s="101">
+        <v>34.4514</v>
+      </c>
+      <c r="C10" s="101">
+        <v>5067</v>
+      </c>
+      <c r="E10" s="98"/>
+      <c r="F10" s="99"/>
+    </row>
+    <row r="11" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A11" s="101">
         <v>3694</v>
       </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="E15">
+      <c r="B11" s="101">
+        <v>34.5837</v>
+      </c>
+      <c r="C11" s="101">
+        <v>5069</v>
+      </c>
+      <c r="E11" s="98"/>
+      <c r="F11" s="99"/>
+    </row>
+    <row r="12" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A12" s="101">
         <v>3757</v>
       </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A16">
-        <v>3681</v>
-      </c>
-      <c r="B16">
-        <v>34</v>
-      </c>
-      <c r="E16">
+      <c r="B12" s="101">
+        <v>34.189700000000002</v>
+      </c>
+      <c r="C12" s="101">
+        <v>5070</v>
+      </c>
+      <c r="E12" s="98"/>
+      <c r="F12" s="99"/>
+    </row>
+    <row r="13" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A13" s="101">
         <v>3758</v>
       </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="E17">
-        <v>3773</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="E18">
-        <v>3774</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="E19">
+      <c r="B13" s="101">
+        <v>34.548099999999998</v>
+      </c>
+      <c r="C13" s="101">
+        <v>5071</v>
+      </c>
+      <c r="E13" s="98"/>
+      <c r="F13" s="99"/>
+    </row>
+    <row r="14" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A14" s="101">
         <v>3786</v>
       </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="E20">
+      <c r="B14" s="101">
+        <v>34.406700000000001</v>
+      </c>
+      <c r="C14" s="101">
+        <v>5572</v>
+      </c>
+      <c r="E14" s="98"/>
+      <c r="F14" s="99"/>
+    </row>
+    <row r="15" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A15" s="101">
         <v>3788</v>
       </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="E21">
+      <c r="B15" s="101">
+        <v>34.795400000000001</v>
+      </c>
+      <c r="C15" s="100">
+        <v>5575</v>
+      </c>
+      <c r="E15" s="98"/>
+      <c r="F15" s="99"/>
+    </row>
+    <row r="16" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A16" s="101">
         <v>3844</v>
       </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="E22">
+      <c r="B16" s="101">
+        <v>34.238300000000002</v>
+      </c>
+      <c r="E16" s="98"/>
+      <c r="F16" s="99"/>
+    </row>
+    <row r="17" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A17" s="101">
         <v>3845</v>
       </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="E23">
+      <c r="B17" s="101">
+        <v>34.294699999999999</v>
+      </c>
+      <c r="C17" s="100"/>
+      <c r="E17" s="98"/>
+      <c r="F17" s="99"/>
+    </row>
+    <row r="18" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A18" s="101">
         <v>3846</v>
       </c>
-      <c r="G23" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="E24">
+      <c r="B18" s="101">
+        <v>34.198399999999999</v>
+      </c>
+      <c r="C18" s="100"/>
+      <c r="E18" s="98"/>
+      <c r="F18" s="99"/>
+    </row>
+    <row r="19" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A19" s="101">
         <v>4003</v>
       </c>
-      <c r="G24" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="E25">
+      <c r="B19" s="101">
+        <v>34.405099999999997</v>
+      </c>
+      <c r="C19" s="100"/>
+      <c r="E19" s="98"/>
+      <c r="F19" s="99"/>
+    </row>
+    <row r="20" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A20" s="101">
         <v>4006</v>
       </c>
-      <c r="G25" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A26" s="98">
-        <v>5082</v>
-      </c>
-      <c r="B26">
-        <v>41</v>
-      </c>
-      <c r="C26" s="98">
-        <v>5071</v>
-      </c>
-      <c r="E26">
+      <c r="B20" s="101">
+        <v>34.403399999999998</v>
+      </c>
+      <c r="C20" s="100"/>
+      <c r="E20" s="98"/>
+      <c r="F20" s="99"/>
+    </row>
+    <row r="21" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A21" s="101">
         <v>4344</v>
       </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A27" s="98">
-        <v>5083</v>
-      </c>
-      <c r="B27">
-        <v>41</v>
-      </c>
-      <c r="E27">
+      <c r="B21" s="101">
+        <v>40.787399999999998</v>
+      </c>
+      <c r="C21" s="100"/>
+      <c r="E21" s="98"/>
+      <c r="F21" s="99"/>
+    </row>
+    <row r="22" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A22" s="101">
         <v>4345</v>
       </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A28" s="98">
-        <v>5176</v>
-      </c>
-      <c r="B28">
-        <v>42</v>
-      </c>
-      <c r="E28">
+      <c r="B22" s="101">
+        <v>40.4544</v>
+      </c>
+      <c r="C22" s="102"/>
+      <c r="E22" s="98"/>
+      <c r="F22" s="99"/>
+    </row>
+    <row r="23" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A23" s="101">
         <v>4400</v>
       </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A29" s="98">
-        <v>5180</v>
-      </c>
-      <c r="B29">
-        <v>42</v>
-      </c>
-      <c r="E29">
+      <c r="B23" s="101">
+        <v>41.503</v>
+      </c>
+      <c r="C23" s="100"/>
+      <c r="E23" s="98"/>
+      <c r="F23" s="99"/>
+    </row>
+    <row r="24" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A24" s="101">
         <v>4722</v>
       </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A30">
+      <c r="B24" s="101">
+        <v>41.790599999999998</v>
+      </c>
+      <c r="C24" s="100"/>
+      <c r="E24" s="98"/>
+      <c r="F24" s="99"/>
+    </row>
+    <row r="25" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A25" s="101">
+        <v>4735</v>
+      </c>
+      <c r="B25" s="101">
+        <v>40.693800000000003</v>
+      </c>
+      <c r="C25" s="100"/>
+      <c r="E25" s="98"/>
+      <c r="F25" s="99"/>
+    </row>
+    <row r="26" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A26" s="101">
+        <v>4926</v>
+      </c>
+      <c r="B26" s="101">
+        <v>40.065600000000003</v>
+      </c>
+      <c r="C26" s="100"/>
+      <c r="E26" s="98"/>
+      <c r="F26" s="99"/>
+    </row>
+    <row r="27" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A27" s="101">
+        <v>4929</v>
+      </c>
+      <c r="B27" s="101">
+        <v>39.681800000000003</v>
+      </c>
+      <c r="C27" s="100"/>
+      <c r="E27" s="98"/>
+      <c r="F27" s="99"/>
+    </row>
+    <row r="28" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A28" s="101">
+        <v>4985</v>
+      </c>
+      <c r="B28" s="101">
+        <v>39.793999999999997</v>
+      </c>
+      <c r="C28" s="100"/>
+      <c r="E28" s="98"/>
+      <c r="F28" s="99"/>
+    </row>
+    <row r="29" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A29" s="101">
+        <v>5066</v>
+      </c>
+      <c r="B29" s="101">
+        <v>40.8249</v>
+      </c>
+      <c r="C29" s="100"/>
+      <c r="E29" s="98"/>
+      <c r="F29" s="99"/>
+    </row>
+    <row r="30" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A30" s="101">
+        <v>5068</v>
+      </c>
+      <c r="B30" s="101">
+        <v>40.5184</v>
+      </c>
+      <c r="C30" s="100"/>
+      <c r="E30" s="98"/>
+      <c r="F30" s="99"/>
+    </row>
+    <row r="31" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A31" s="101">
+        <v>5290</v>
+      </c>
+      <c r="B31" s="101">
+        <v>40.1541</v>
+      </c>
+      <c r="C31" s="100"/>
+      <c r="E31" s="98"/>
+      <c r="F31" s="99"/>
+    </row>
+    <row r="32" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A32" s="101">
+        <v>5292</v>
+      </c>
+      <c r="B32" s="101">
+        <v>39.639899999999997</v>
+      </c>
+      <c r="C32" s="100"/>
+      <c r="E32" s="98"/>
+      <c r="F32" s="99"/>
+    </row>
+    <row r="33" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A33" s="101">
+        <v>5294</v>
+      </c>
+      <c r="B33" s="101">
+        <v>39.4373</v>
+      </c>
+      <c r="C33" s="100"/>
+      <c r="E33" s="98"/>
+      <c r="F33" s="99"/>
+    </row>
+    <row r="34" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A34" s="101">
+        <v>5322</v>
+      </c>
+      <c r="B34" s="101">
+        <v>29.418900000000001</v>
+      </c>
+      <c r="C34" s="100"/>
+      <c r="E34" s="98"/>
+      <c r="F34" s="99"/>
+    </row>
+    <row r="35" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A35" s="101">
+        <v>5423</v>
+      </c>
+      <c r="B35" s="101">
+        <v>39.663800000000002</v>
+      </c>
+      <c r="C35" s="100"/>
+      <c r="E35" s="98"/>
+      <c r="F35" s="99"/>
+    </row>
+    <row r="36" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A36" s="101">
         <v>5710</v>
       </c>
-      <c r="B30">
-        <v>30</v>
-      </c>
-      <c r="E30">
-        <v>4735</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="E31">
-        <v>4926</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="E32">
-        <v>4929</v>
-      </c>
-    </row>
-    <row r="33" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E33">
-        <v>4985</v>
-      </c>
-    </row>
-    <row r="34" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E34">
-        <v>5066</v>
-      </c>
-    </row>
-    <row r="35" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E35">
-        <v>5067</v>
-      </c>
-    </row>
-    <row r="36" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E36">
-        <v>5068</v>
-      </c>
-    </row>
-    <row r="37" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E37">
-        <v>5069</v>
-      </c>
-    </row>
-    <row r="38" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E38">
-        <v>5070</v>
-      </c>
-    </row>
-    <row r="39" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E39">
-        <v>5071</v>
-      </c>
-    </row>
-    <row r="40" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E40">
-        <v>5290</v>
-      </c>
-    </row>
-    <row r="41" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E41">
-        <v>5292</v>
-      </c>
-    </row>
-    <row r="42" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E42">
-        <v>5294</v>
-      </c>
-    </row>
-    <row r="43" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E43">
-        <v>5322</v>
-      </c>
+      <c r="B36" s="101">
+        <v>31.2072</v>
+      </c>
+      <c r="C36" s="100"/>
+      <c r="E36" s="98"/>
+      <c r="F36" s="99"/>
+    </row>
+    <row r="37" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A37" s="101">
+        <v>5722</v>
+      </c>
+      <c r="B37" s="101">
+        <v>31.4803</v>
+      </c>
+      <c r="C37" s="100"/>
+      <c r="E37" s="98"/>
+      <c r="F37" s="99"/>
+    </row>
+    <row r="38" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A38" s="101">
+        <v>5723</v>
+      </c>
+      <c r="B38" s="101">
+        <v>31.637499999999999</v>
+      </c>
+      <c r="C38" s="100"/>
+      <c r="E38" s="98"/>
+      <c r="F38" s="99"/>
+    </row>
+    <row r="39" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A39" s="101">
+        <v>5724</v>
+      </c>
+      <c r="B39" s="101">
+        <v>31.4101</v>
+      </c>
+      <c r="C39" s="100"/>
+      <c r="E39" s="98"/>
+      <c r="F39" s="99"/>
+    </row>
+    <row r="40" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A40" s="101">
+        <v>5726</v>
+      </c>
+      <c r="B40" s="101">
+        <v>31.5975</v>
+      </c>
+      <c r="C40" s="100"/>
+      <c r="E40" s="98"/>
+      <c r="F40" s="99"/>
+    </row>
+    <row r="41" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A41" s="101">
+        <v>5794</v>
+      </c>
+      <c r="B41" s="101">
+        <v>31.710899999999999</v>
+      </c>
+      <c r="E41" s="98"/>
+      <c r="F41" s="99"/>
+    </row>
+    <row r="42" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A42" s="101">
+        <v>5795</v>
+      </c>
+      <c r="B42" s="101">
+        <v>31.599900000000002</v>
+      </c>
+      <c r="E42" s="98"/>
+      <c r="F42" s="99"/>
+    </row>
+    <row r="43" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A43" s="101">
+        <v>5976</v>
+      </c>
+      <c r="B43" s="101">
+        <v>28.605399999999999</v>
+      </c>
+      <c r="E43" s="98"/>
+      <c r="F43" s="99"/>
+    </row>
+    <row r="44" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A44" s="101">
+        <v>5979</v>
+      </c>
+      <c r="B44" s="101">
+        <v>29.110900000000001</v>
+      </c>
+      <c r="E44" s="98"/>
+      <c r="F44" s="99"/>
+    </row>
+    <row r="45" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A45" s="101">
+        <v>5992</v>
+      </c>
+      <c r="B45" s="101">
+        <v>28.8826</v>
+      </c>
+      <c r="E45" s="98"/>
+      <c r="F45" s="99"/>
+    </row>
+    <row r="46" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A46" s="100">
+        <v>5795</v>
+      </c>
+      <c r="E46" s="98"/>
+      <c r="F46" s="99"/>
+    </row>
+    <row r="47" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A47" s="100">
+        <v>5976</v>
+      </c>
+      <c r="E47" s="98"/>
+      <c r="F47" s="99"/>
+    </row>
+    <row r="48" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A48" s="100">
+        <v>5979</v>
+      </c>
+      <c r="E48" s="98"/>
+      <c r="F48" s="99"/>
+    </row>
+    <row r="49" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A49" s="100">
+        <v>5992</v>
+      </c>
+      <c r="E49" s="98"/>
+      <c r="F49" s="99"/>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="E50" s="98"/>
+      <c r="F50" s="99"/>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="E51" s="98"/>
+      <c r="F51" s="99"/>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="E52" s="98"/>
+      <c r="F52" s="99"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1366,14 +1650,14 @@
       </c>
       <c r="C1" s="2"/>
       <c r="D1" s="3"/>
-      <c r="E1" s="87" t="s">
+      <c r="E1" s="96" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="88"/>
-      <c r="G1" s="88"/>
-      <c r="H1" s="88"/>
-      <c r="I1" s="88"/>
-      <c r="J1" s="88"/>
+      <c r="F1" s="97"/>
+      <c r="G1" s="97"/>
+      <c r="H1" s="97"/>
+      <c r="I1" s="97"/>
+      <c r="J1" s="97"/>
       <c r="K1" s="4" t="s">
         <v>2</v>
       </c>
@@ -4038,72 +4322,72 @@
       <c r="AQ39" s="10"/>
       <c r="AR39" s="10"/>
     </row>
-    <row r="40" spans="1:44" s="97" customFormat="1" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="89">
+    <row r="40" spans="1:44" s="95" customFormat="1" ht="13" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A40" s="87">
         <v>5071</v>
       </c>
-      <c r="B40" s="90">
+      <c r="B40" s="88">
         <v>45840</v>
       </c>
-      <c r="C40" s="91"/>
-      <c r="D40" s="92" t="s">
+      <c r="C40" s="89"/>
+      <c r="D40" s="90" t="s">
         <v>90</v>
       </c>
-      <c r="E40" s="93" t="s">
+      <c r="E40" s="91" t="s">
         <v>48</v>
       </c>
-      <c r="F40" s="92">
+      <c r="F40" s="90">
         <v>5</v>
       </c>
-      <c r="G40" s="94">
+      <c r="G40" s="92">
         <v>1756.6</v>
       </c>
-      <c r="H40" s="94">
+      <c r="H40" s="92">
         <v>1762.2</v>
       </c>
-      <c r="I40" s="95">
+      <c r="I40" s="93">
         <v>0.6</v>
       </c>
-      <c r="J40" s="95">
+      <c r="J40" s="93">
         <v>0.2</v>
       </c>
-      <c r="K40" s="93" t="s">
+      <c r="K40" s="91" t="s">
         <v>84</v>
       </c>
-      <c r="L40" s="96"/>
-      <c r="M40" s="92"/>
-      <c r="N40" s="92"/>
-      <c r="O40" s="92"/>
-      <c r="Q40" s="92"/>
-      <c r="R40" s="92"/>
-      <c r="S40" s="92" t="s">
+      <c r="L40" s="94"/>
+      <c r="M40" s="90"/>
+      <c r="N40" s="90"/>
+      <c r="O40" s="90"/>
+      <c r="Q40" s="90"/>
+      <c r="R40" s="90"/>
+      <c r="S40" s="90" t="s">
         <v>72</v>
       </c>
-      <c r="T40" s="92"/>
-      <c r="U40" s="92"/>
-      <c r="V40" s="92"/>
-      <c r="W40" s="92"/>
-      <c r="X40" s="92"/>
-      <c r="Y40" s="92"/>
-      <c r="Z40" s="92"/>
-      <c r="AA40" s="92"/>
-      <c r="AB40" s="92"/>
-      <c r="AC40" s="92"/>
-      <c r="AD40" s="92"/>
-      <c r="AE40" s="92"/>
-      <c r="AF40" s="92"/>
-      <c r="AG40" s="92"/>
-      <c r="AH40" s="92"/>
-      <c r="AI40" s="92"/>
-      <c r="AJ40" s="92"/>
-      <c r="AK40" s="92"/>
-      <c r="AL40" s="92"/>
-      <c r="AM40" s="92"/>
-      <c r="AN40" s="92"/>
-      <c r="AO40" s="92"/>
-      <c r="AP40" s="92"/>
-      <c r="AQ40" s="92"/>
-      <c r="AR40" s="92"/>
+      <c r="T40" s="90"/>
+      <c r="U40" s="90"/>
+      <c r="V40" s="90"/>
+      <c r="W40" s="90"/>
+      <c r="X40" s="90"/>
+      <c r="Y40" s="90"/>
+      <c r="Z40" s="90"/>
+      <c r="AA40" s="90"/>
+      <c r="AB40" s="90"/>
+      <c r="AC40" s="90"/>
+      <c r="AD40" s="90"/>
+      <c r="AE40" s="90"/>
+      <c r="AF40" s="90"/>
+      <c r="AG40" s="90"/>
+      <c r="AH40" s="90"/>
+      <c r="AI40" s="90"/>
+      <c r="AJ40" s="90"/>
+      <c r="AK40" s="90"/>
+      <c r="AL40" s="90"/>
+      <c r="AM40" s="90"/>
+      <c r="AN40" s="90"/>
+      <c r="AO40" s="90"/>
+      <c r="AP40" s="90"/>
+      <c r="AQ40" s="90"/>
+      <c r="AR40" s="90"/>
     </row>
     <row r="41" spans="1:44" ht="13" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="21">
@@ -4899,14 +5183,14 @@
       </c>
       <c r="C1" s="2"/>
       <c r="D1" s="3"/>
-      <c r="E1" s="87" t="s">
+      <c r="E1" s="96" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="88"/>
-      <c r="G1" s="88"/>
-      <c r="H1" s="88"/>
-      <c r="I1" s="88"/>
-      <c r="J1" s="88"/>
+      <c r="F1" s="97"/>
+      <c r="G1" s="97"/>
+      <c r="H1" s="97"/>
+      <c r="I1" s="97"/>
+      <c r="J1" s="97"/>
       <c r="K1" s="4" t="s">
         <v>2</v>
       </c>

</xml_diff>